<commit_message>
Update analysis scripts, results, and data across DiD, SDID, and flow analyses
Substantial revisions to descriptives, DiD, SDID, flow, individual, and revenue
analysis code. Add new scripts (elasticities, narrow SDID, quarterly SDID,
appendix data quality). Update figures, tables, maps, and data.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Table2.xlsx
+++ b/results/Table2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="441" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="2499" uniqueCount="29">
   <si>
     <t>state_name</t>
   </si>
@@ -920,25 +920,25 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D6" s="1">
-        <v>0.043668478727340698</v>
+        <v>0.041713923215866089</v>
       </c>
       <c r="E6" s="1">
-        <v>0.040553078055381775</v>
+        <v>0.040620841085910797</v>
       </c>
       <c r="F6" s="1">
-        <v>0.034268669784069061</v>
+        <v>0.034140396863222122</v>
       </c>
       <c r="G6" s="1">
-        <v>0.034138523042201996</v>
+        <v>0.036069039255380631</v>
       </c>
       <c r="H6" s="1">
-        <v>0.046879116445779801</v>
+        <v>0.043224930763244629</v>
       </c>
       <c r="I6" s="1">
-        <v>0.041988909244537354</v>
+        <v>0.045515932142734528</v>
       </c>
     </row>
     <row r="7">
@@ -949,25 +949,25 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D7" s="1">
-        <v>0.041713923215866089</v>
+        <v>0.043668478727340698</v>
       </c>
       <c r="E7" s="1">
-        <v>0.040620841085910797</v>
+        <v>0.040553078055381775</v>
       </c>
       <c r="F7" s="1">
-        <v>0.034140396863222122</v>
+        <v>0.034268669784069061</v>
       </c>
       <c r="G7" s="1">
-        <v>0.036069039255380631</v>
+        <v>0.034138523042201996</v>
       </c>
       <c r="H7" s="1">
-        <v>0.043224930763244629</v>
+        <v>0.046879116445779801</v>
       </c>
       <c r="I7" s="1">
-        <v>0.045515932142734528</v>
+        <v>0.041988909244537354</v>
       </c>
     </row>
     <row r="8">
@@ -1007,25 +1007,25 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D9" s="1">
-        <v>0.066813893616199493</v>
+        <v>0.078097611665725708</v>
       </c>
       <c r="E9" s="1">
-        <v>0.057924751192331314</v>
+        <v>0.06375441700220108</v>
       </c>
       <c r="F9" s="1">
-        <v>0.062374264001846313</v>
+        <v>0.072186104953289032</v>
       </c>
       <c r="G9" s="1">
-        <v>0.047444775700569153</v>
+        <v>0.048510834574699402</v>
       </c>
       <c r="H9" s="1">
-        <v>0.078170418739318848</v>
+        <v>0.08697471022605896</v>
       </c>
       <c r="I9" s="1">
-        <v>0.052892241626977921</v>
+        <v>0.059970732778310776</v>
       </c>
     </row>
     <row r="10">
@@ -1036,25 +1036,25 @@
         <v>7</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D10" s="1">
-        <v>0.078097611665725708</v>
+        <v>0.066813893616199493</v>
       </c>
       <c r="E10" s="1">
-        <v>0.06375441700220108</v>
+        <v>0.057924751192331314</v>
       </c>
       <c r="F10" s="1">
-        <v>0.072186104953289032</v>
+        <v>0.062374264001846313</v>
       </c>
       <c r="G10" s="1">
-        <v>0.048510834574699402</v>
+        <v>0.047444775700569153</v>
       </c>
       <c r="H10" s="1">
-        <v>0.08697471022605896</v>
+        <v>0.078170418739318848</v>
       </c>
       <c r="I10" s="1">
-        <v>0.059970732778310776</v>
+        <v>0.052892241626977921</v>
       </c>
     </row>
     <row r="11">
@@ -1094,25 +1094,25 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D12" s="1">
-        <v>0.039367526769638062</v>
+        <v>0.045784421265125275</v>
       </c>
       <c r="E12" s="1">
-        <v>0.04078688845038414</v>
+        <v>0.039934225380420685</v>
       </c>
       <c r="F12" s="1">
-        <v>0.036130271852016449</v>
+        <v>0.041493140161037445</v>
       </c>
       <c r="G12" s="1">
-        <v>0.036443993449211121</v>
+        <v>0.035399135202169418</v>
       </c>
       <c r="H12" s="1">
-        <v>0.047341573983430862</v>
+        <v>0.056529216468334198</v>
       </c>
       <c r="I12" s="1">
-        <v>0.05091317743062973</v>
+        <v>0.051557201892137528</v>
       </c>
     </row>
     <row r="13">
@@ -1123,25 +1123,25 @@
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D13" s="1">
-        <v>0.045784421265125275</v>
+        <v>0.039367526769638062</v>
       </c>
       <c r="E13" s="1">
-        <v>0.039934225380420685</v>
+        <v>0.04078688845038414</v>
       </c>
       <c r="F13" s="1">
-        <v>0.041493140161037445</v>
+        <v>0.036130271852016449</v>
       </c>
       <c r="G13" s="1">
-        <v>0.035399135202169418</v>
+        <v>0.036443993449211121</v>
       </c>
       <c r="H13" s="1">
-        <v>0.056529216468334198</v>
+        <v>0.047341573983430862</v>
       </c>
       <c r="I13" s="1">
-        <v>0.051557201892137528</v>
+        <v>0.05091317743062973</v>
       </c>
     </row>
     <row r="14">
@@ -1181,25 +1181,25 @@
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D15" s="1">
-        <v>0.059178154915571213</v>
+        <v>0.070727154612541199</v>
       </c>
       <c r="E15" s="1">
-        <v>0.056496087461709976</v>
+        <v>0.064735077321529388</v>
       </c>
       <c r="F15" s="1">
-        <v>0.052232503890991211</v>
+        <v>0.064169019460678101</v>
       </c>
       <c r="G15" s="1">
-        <v>0.044814392924308777</v>
+        <v>0.049849245697259903</v>
       </c>
       <c r="H15" s="1">
-        <v>0.054016690701246262</v>
+        <v>0.068740174174308777</v>
       </c>
       <c r="I15" s="1">
-        <v>0.052172701805830002</v>
+        <v>0.056195486336946488</v>
       </c>
     </row>
     <row r="16">
@@ -1210,25 +1210,25 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D16" s="1">
-        <v>0.070727154612541199</v>
+        <v>0.059178154915571213</v>
       </c>
       <c r="E16" s="1">
-        <v>0.064735077321529388</v>
+        <v>0.056496087461709976</v>
       </c>
       <c r="F16" s="1">
-        <v>0.064169019460678101</v>
+        <v>0.052232503890991211</v>
       </c>
       <c r="G16" s="1">
-        <v>0.049849245697259903</v>
+        <v>0.044814392924308777</v>
       </c>
       <c r="H16" s="1">
-        <v>0.068740174174308777</v>
+        <v>0.054016690701246262</v>
       </c>
       <c r="I16" s="1">
-        <v>0.056195486336946488</v>
+        <v>0.052172701805830002</v>
       </c>
     </row>
     <row r="17">
@@ -1239,25 +1239,25 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D17" s="1">
-        <v>0.040310077369213104</v>
+        <v>0.041196983307600021</v>
       </c>
       <c r="E17" s="1">
-        <v>0.067308209836483002</v>
+        <v>0.059329647570848465</v>
       </c>
       <c r="F17" s="1">
-        <v>0.034843768924474716</v>
+        <v>0.03178974986076355</v>
       </c>
       <c r="G17" s="1">
-        <v>0.070556610822677612</v>
+        <v>0.050676636397838593</v>
       </c>
       <c r="H17" s="1">
-        <v>0.067878447473049164</v>
+        <v>0.046695537865161896</v>
       </c>
       <c r="I17" s="1">
-        <v>0.098924554884433746</v>
+        <v>0.071552000939846039</v>
       </c>
     </row>
     <row r="18">
@@ -1268,25 +1268,25 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D18" s="1">
-        <v>0.041196983307600021</v>
+        <v>0.040310077369213104</v>
       </c>
       <c r="E18" s="1">
-        <v>0.059329647570848465</v>
+        <v>0.067308209836483002</v>
       </c>
       <c r="F18" s="1">
-        <v>0.03178974986076355</v>
+        <v>0.034843768924474716</v>
       </c>
       <c r="G18" s="1">
-        <v>0.050676636397838593</v>
+        <v>0.070556610822677612</v>
       </c>
       <c r="H18" s="1">
-        <v>0.046695537865161896</v>
+        <v>0.067878447473049164</v>
       </c>
       <c r="I18" s="1">
-        <v>0.071552000939846039</v>
+        <v>0.098924554884433746</v>
       </c>
     </row>
     <row r="19">
@@ -1326,25 +1326,25 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D20" s="1">
-        <v>0.047015395015478134</v>
+        <v>0.04233773797750473</v>
       </c>
       <c r="E20" s="1">
-        <v>0.061984565109014511</v>
+        <v>0.054828748106956482</v>
       </c>
       <c r="F20" s="1">
-        <v>0.04625726118683815</v>
+        <v>0.039202205836772919</v>
       </c>
       <c r="G20" s="1">
-        <v>0.057423654943704605</v>
+        <v>0.049602121114730835</v>
       </c>
       <c r="H20" s="1">
-        <v>0.050053652375936508</v>
+        <v>0.043669760227203369</v>
       </c>
       <c r="I20" s="1">
-        <v>0.082157902419567108</v>
+        <v>0.072661422193050385</v>
       </c>
     </row>
     <row r="21">
@@ -1355,25 +1355,25 @@
         <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D21" s="1">
-        <v>0.04233773797750473</v>
+        <v>0.047015395015478134</v>
       </c>
       <c r="E21" s="1">
-        <v>0.054828748106956482</v>
+        <v>0.061984565109014511</v>
       </c>
       <c r="F21" s="1">
-        <v>0.039202205836772919</v>
+        <v>0.04625726118683815</v>
       </c>
       <c r="G21" s="1">
-        <v>0.049602121114730835</v>
+        <v>0.057423654943704605</v>
       </c>
       <c r="H21" s="1">
-        <v>0.043669760227203369</v>
+        <v>0.050053652375936508</v>
       </c>
       <c r="I21" s="1">
-        <v>0.072661422193050385</v>
+        <v>0.082157902419567108</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Refactor IRS migration pipeline, add SDID influence/speccurve plots, clean temp files
Major changes:
- Refactor 01f_irs_migration.do (consolidate year-range globals in 00_multnomah.do)
- Add setup_parallel program in 01a_programs.do for standalone execution
- Add SDID influence coefficient and spec curve (outstate) figures
- Remove old SDID temp_results .dta files (now gitignored)
- Add results/flows/temp_results/ to .gitignore
- Update R/api_code.R and all downstream results/figures

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/Table2.xlsx
+++ b/results/Table2.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="2499" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="3087" uniqueCount="29">
   <si>
     <t>state_name</t>
   </si>
@@ -920,25 +920,25 @@
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D6" s="1">
-        <v>0.041713923215866089</v>
+        <v>0.043668478727340698</v>
       </c>
       <c r="E6" s="1">
-        <v>0.040620841085910797</v>
+        <v>0.040553078055381775</v>
       </c>
       <c r="F6" s="1">
-        <v>0.034140396863222122</v>
+        <v>0.034268669784069061</v>
       </c>
       <c r="G6" s="1">
-        <v>0.036069039255380631</v>
+        <v>0.034138523042201996</v>
       </c>
       <c r="H6" s="1">
-        <v>0.043224930763244629</v>
+        <v>0.046879116445779801</v>
       </c>
       <c r="I6" s="1">
-        <v>0.045515932142734528</v>
+        <v>0.041988909244537354</v>
       </c>
     </row>
     <row r="7">
@@ -949,25 +949,25 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D7" s="1">
-        <v>0.043668478727340698</v>
+        <v>0.041713923215866089</v>
       </c>
       <c r="E7" s="1">
-        <v>0.040553078055381775</v>
+        <v>0.040620841085910797</v>
       </c>
       <c r="F7" s="1">
-        <v>0.034268669784069061</v>
+        <v>0.034140396863222122</v>
       </c>
       <c r="G7" s="1">
-        <v>0.034138523042201996</v>
+        <v>0.036069039255380631</v>
       </c>
       <c r="H7" s="1">
-        <v>0.046879116445779801</v>
+        <v>0.043224930763244629</v>
       </c>
       <c r="I7" s="1">
-        <v>0.041988909244537354</v>
+        <v>0.045515932142734528</v>
       </c>
     </row>
     <row r="8">
@@ -1094,25 +1094,25 @@
         <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D12" s="1">
-        <v>0.045784421265125275</v>
+        <v>0.039367526769638062</v>
       </c>
       <c r="E12" s="1">
-        <v>0.039934225380420685</v>
+        <v>0.04078688845038414</v>
       </c>
       <c r="F12" s="1">
-        <v>0.041493140161037445</v>
+        <v>0.036130271852016449</v>
       </c>
       <c r="G12" s="1">
-        <v>0.035399135202169418</v>
+        <v>0.036443993449211121</v>
       </c>
       <c r="H12" s="1">
-        <v>0.056529216468334198</v>
+        <v>0.047341573983430862</v>
       </c>
       <c r="I12" s="1">
-        <v>0.051557201892137528</v>
+        <v>0.05091317743062973</v>
       </c>
     </row>
     <row r="13">
@@ -1123,25 +1123,25 @@
         <v>8</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D13" s="1">
-        <v>0.039367526769638062</v>
+        <v>0.045784421265125275</v>
       </c>
       <c r="E13" s="1">
-        <v>0.04078688845038414</v>
+        <v>0.039934225380420685</v>
       </c>
       <c r="F13" s="1">
-        <v>0.036130271852016449</v>
+        <v>0.041493140161037445</v>
       </c>
       <c r="G13" s="1">
-        <v>0.036443993449211121</v>
+        <v>0.035399135202169418</v>
       </c>
       <c r="H13" s="1">
-        <v>0.047341573983430862</v>
+        <v>0.056529216468334198</v>
       </c>
       <c r="I13" s="1">
-        <v>0.05091317743062973</v>
+        <v>0.051557201892137528</v>
       </c>
     </row>
     <row r="14">
@@ -1181,25 +1181,25 @@
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D15" s="1">
-        <v>0.070727154612541199</v>
+        <v>0.059178154915571213</v>
       </c>
       <c r="E15" s="1">
-        <v>0.064735077321529388</v>
+        <v>0.056496087461709976</v>
       </c>
       <c r="F15" s="1">
-        <v>0.064169019460678101</v>
+        <v>0.052232503890991211</v>
       </c>
       <c r="G15" s="1">
-        <v>0.049849245697259903</v>
+        <v>0.044814392924308777</v>
       </c>
       <c r="H15" s="1">
-        <v>0.068740174174308777</v>
+        <v>0.054016690701246262</v>
       </c>
       <c r="I15" s="1">
-        <v>0.056195486336946488</v>
+        <v>0.052172701805830002</v>
       </c>
     </row>
     <row r="16">
@@ -1210,25 +1210,25 @@
         <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D16" s="1">
-        <v>0.059178154915571213</v>
+        <v>0.070727154612541199</v>
       </c>
       <c r="E16" s="1">
-        <v>0.056496087461709976</v>
+        <v>0.064735077321529388</v>
       </c>
       <c r="F16" s="1">
-        <v>0.052232503890991211</v>
+        <v>0.064169019460678101</v>
       </c>
       <c r="G16" s="1">
-        <v>0.044814392924308777</v>
+        <v>0.049849245697259903</v>
       </c>
       <c r="H16" s="1">
-        <v>0.054016690701246262</v>
+        <v>0.068740174174308777</v>
       </c>
       <c r="I16" s="1">
-        <v>0.052172701805830002</v>
+        <v>0.056195486336946488</v>
       </c>
     </row>
     <row r="17">
@@ -1239,25 +1239,25 @@
         <v>10</v>
       </c>
       <c r="C17" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D17" s="1">
-        <v>0.041196983307600021</v>
+        <v>0.040310077369213104</v>
       </c>
       <c r="E17" s="1">
-        <v>0.059329647570848465</v>
+        <v>0.067308209836483002</v>
       </c>
       <c r="F17" s="1">
-        <v>0.03178974986076355</v>
+        <v>0.034843768924474716</v>
       </c>
       <c r="G17" s="1">
-        <v>0.050676636397838593</v>
+        <v>0.070556610822677612</v>
       </c>
       <c r="H17" s="1">
-        <v>0.046695537865161896</v>
+        <v>0.067878447473049164</v>
       </c>
       <c r="I17" s="1">
-        <v>0.071552000939846039</v>
+        <v>0.098924554884433746</v>
       </c>
     </row>
     <row r="18">
@@ -1268,25 +1268,25 @@
         <v>10</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D18" s="1">
-        <v>0.040310077369213104</v>
+        <v>0.041196983307600021</v>
       </c>
       <c r="E18" s="1">
-        <v>0.067308209836483002</v>
+        <v>0.059329647570848465</v>
       </c>
       <c r="F18" s="1">
-        <v>0.034843768924474716</v>
+        <v>0.03178974986076355</v>
       </c>
       <c r="G18" s="1">
-        <v>0.070556610822677612</v>
+        <v>0.050676636397838593</v>
       </c>
       <c r="H18" s="1">
-        <v>0.067878447473049164</v>
+        <v>0.046695537865161896</v>
       </c>
       <c r="I18" s="1">
-        <v>0.098924554884433746</v>
+        <v>0.071552000939846039</v>
       </c>
     </row>
     <row r="19">
@@ -1326,25 +1326,25 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="D20" s="1">
-        <v>0.04233773797750473</v>
+        <v>0.047015395015478134</v>
       </c>
       <c r="E20" s="1">
-        <v>0.054828748106956482</v>
+        <v>0.061984565109014511</v>
       </c>
       <c r="F20" s="1">
-        <v>0.039202205836772919</v>
+        <v>0.04625726118683815</v>
       </c>
       <c r="G20" s="1">
-        <v>0.049602121114730835</v>
+        <v>0.057423654943704605</v>
       </c>
       <c r="H20" s="1">
-        <v>0.043669760227203369</v>
+        <v>0.050053652375936508</v>
       </c>
       <c r="I20" s="1">
-        <v>0.072661422193050385</v>
+        <v>0.082157902419567108</v>
       </c>
     </row>
     <row r="21">
@@ -1355,25 +1355,25 @@
         <v>11</v>
       </c>
       <c r="C21" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="D21" s="1">
-        <v>0.047015395015478134</v>
+        <v>0.04233773797750473</v>
       </c>
       <c r="E21" s="1">
-        <v>0.061984565109014511</v>
+        <v>0.054828748106956482</v>
       </c>
       <c r="F21" s="1">
-        <v>0.04625726118683815</v>
+        <v>0.039202205836772919</v>
       </c>
       <c r="G21" s="1">
-        <v>0.057423654943704605</v>
+        <v>0.049602121114730835</v>
       </c>
       <c r="H21" s="1">
-        <v>0.050053652375936508</v>
+        <v>0.043669760227203369</v>
       </c>
       <c r="I21" s="1">
-        <v>0.082157902419567108</v>
+        <v>0.072661422193050385</v>
       </c>
     </row>
     <row r="22">

</xml_diff>